<commit_message>
sn: add ia senegal
</commit_message>
<xml_diff>
--- a/SCH-STH/Impact assessments/Senegal/2025/octobre/sn_sppa_impact_2510_4_qualite.xlsx
+++ b/SCH-STH/Impact assessments/Senegal/2025/octobre/sn_sppa_impact_2510_4_qualite.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yumbad\Repositories\dsa-forms\SCH-STH\Impact assessments\Senegal\2025\octobre\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2323E15C-17C9-4463-9B6B-74E1D7C960C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1382D9C5-DE0B-4446-B9DA-5814B2B3E290}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="survey" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="358" uniqueCount="216">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="356" uniqueCount="214">
   <si>
     <t>type</t>
   </si>
@@ -565,12 +565,6 @@
   </si>
   <si>
     <t>Ce code a déjà été sélectionné.</t>
-  </si>
-  <si>
-    <t>. = 'FATICK' or . = 'KHOMBOLE'</t>
-  </si>
-  <si>
-    <t>Fatick et Khombole uniquement</t>
   </si>
   <si>
     <t>${q_autre_nom_1} nombre d'oeufs lame A</t>
@@ -1504,7 +1498,7 @@
       <c r="S3" s="16"/>
       <c r="T3" s="16"/>
     </row>
-    <row r="4" spans="1:20" s="5" customFormat="1" ht="30">
+    <row r="4" spans="1:20" s="5" customFormat="1">
       <c r="A4" s="35" t="s">
         <v>13</v>
       </c>
@@ -1516,12 +1510,8 @@
       </c>
       <c r="D4" s="39"/>
       <c r="E4" s="35"/>
-      <c r="F4" s="40" t="s">
-        <v>181</v>
-      </c>
-      <c r="G4" s="39" t="s">
-        <v>182</v>
-      </c>
+      <c r="F4" s="40"/>
+      <c r="G4" s="39"/>
       <c r="H4" s="35"/>
       <c r="I4" s="35"/>
       <c r="J4" s="35" t="s">
@@ -1679,7 +1669,7 @@
         <v>55</v>
       </c>
       <c r="B9" s="48" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="C9" s="49" t="s">
         <v>60</v>
@@ -1764,13 +1754,13 @@
     </row>
     <row r="12" spans="1:20" s="8" customFormat="1">
       <c r="A12" s="31" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="B12" s="31" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="C12" s="32" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="D12" s="32"/>
       <c r="E12" s="32"/>
@@ -1797,17 +1787,17 @@
         <v>14</v>
       </c>
       <c r="B13" s="34" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="C13" s="34" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="D13" s="34"/>
       <c r="E13" s="34"/>
       <c r="F13" s="34"/>
       <c r="G13" s="34"/>
       <c r="H13" s="31" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="I13" s="32"/>
       <c r="J13" s="34" t="s">
@@ -1829,21 +1819,21 @@
         <v>14</v>
       </c>
       <c r="B14" s="34" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="C14" s="34" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="D14" s="34"/>
       <c r="E14" s="34"/>
       <c r="F14" s="34" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="G14" s="34" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="H14" s="31" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="I14" s="32"/>
       <c r="J14" s="34" t="s">
@@ -1862,22 +1852,22 @@
     </row>
     <row r="15" spans="1:20" s="8" customFormat="1">
       <c r="A15" s="34" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="B15" s="34" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="C15" s="34" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="D15" s="34"/>
       <c r="E15" s="34"/>
       <c r="F15" s="34"/>
       <c r="G15" s="34" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="H15" s="31" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="I15" s="32"/>
       <c r="J15" s="34" t="s">
@@ -1916,7 +1906,7 @@
       </c>
       <c r="H16" s="35"/>
       <c r="I16" s="35" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="J16" s="35" t="s">
         <v>12</v>
@@ -3046,7 +3036,7 @@
         <v>170</v>
       </c>
       <c r="C54" s="11" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="D54" s="11"/>
       <c r="E54" s="28"/>
@@ -3078,7 +3068,7 @@
         <v>171</v>
       </c>
       <c r="C55" s="11" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="D55" s="11"/>
       <c r="E55" s="28"/>
@@ -3107,10 +3097,10 @@
         <v>15</v>
       </c>
       <c r="B56" s="15" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="C56" s="11" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="D56" s="11" t="s">
         <v>47</v>
@@ -3122,7 +3112,7 @@
         <v>169</v>
       </c>
       <c r="I56" s="28" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="J56" s="15" t="s">
         <v>12</v>
@@ -3202,7 +3192,7 @@
         <v>174</v>
       </c>
       <c r="C59" s="11" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="D59" s="12"/>
       <c r="E59" s="16"/>
@@ -3234,7 +3224,7 @@
         <v>175</v>
       </c>
       <c r="C60" s="11" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="D60" s="12"/>
       <c r="E60" s="16"/>
@@ -3263,10 +3253,10 @@
         <v>15</v>
       </c>
       <c r="B61" s="15" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="C61" s="11" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="D61" s="12" t="s">
         <v>47</v>
@@ -3278,7 +3268,7 @@
         <v>173</v>
       </c>
       <c r="I61" s="28" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="J61" s="15" t="s">
         <v>12</v>
@@ -3629,26 +3619,26 @@
     </row>
     <row r="20" spans="1:5">
       <c r="A20" s="64" t="s">
+        <v>208</v>
+      </c>
+      <c r="B20" s="64" t="s">
+        <v>209</v>
+      </c>
+      <c r="C20" s="23" t="s">
         <v>210</v>
-      </c>
-      <c r="B20" s="64" t="s">
-        <v>211</v>
-      </c>
-      <c r="C20" s="23" t="s">
-        <v>212</v>
       </c>
       <c r="D20" s="64"/>
       <c r="E20" s="22"/>
     </row>
     <row r="21" spans="1:5">
       <c r="A21" s="64" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="B21" s="64" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="C21" s="23" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="D21" s="64"/>
       <c r="E21" s="22"/>
@@ -3681,10 +3671,10 @@
     </row>
     <row r="2" spans="1:3">
       <c r="A2" s="8" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="C2" t="s">
         <v>27</v>

</xml_diff>